<commit_message>
Use real delivering battalion names (Gadsar, 699)
Co-Authored-By: Claude Fable 5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01HWaTxciq62ssoxtUxBkqgK
</commit_message>
<xml_diff>
--- a/equipment_handover.xlsx
+++ b/equipment_handover.xlsx
@@ -14,7 +14,7 @@
     <sheet name="מקרא והוראות" sheetId="5" state="visible" r:id="rId5"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm.Print_Area" localSheetId="3">'סיכום וחתימות'!$A$1:$F$53</definedName>
+    <definedName name="_xlnm.Print_Area" localSheetId="3">'סיכום וחתימות'!$A$1:$F$52</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -9066,7 +9066,7 @@
       </c>
       <c r="B3" s="7" t="inlineStr">
         <is>
-          <t>גדוד א׳</t>
+          <t>גדס"ר</t>
         </is>
       </c>
       <c r="C3" s="6" t="n"/>
@@ -9085,7 +9085,7 @@
       </c>
       <c r="B4" s="7" t="inlineStr">
         <is>
-          <t>גדוד א׳</t>
+          <t>גדס"ר</t>
         </is>
       </c>
       <c r="C4" s="6" t="n"/>
@@ -9104,7 +9104,7 @@
       </c>
       <c r="B5" s="7" t="inlineStr">
         <is>
-          <t>גדוד ב׳</t>
+          <t>699</t>
         </is>
       </c>
       <c r="C5" s="6" t="n"/>
@@ -9323,7 +9323,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
-  <dimension ref="A1:F53"/>
+  <dimension ref="A1:F52"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="26" customWidth="1" min="1" max="1"/>
@@ -9360,7 +9360,7 @@
     <row r="5">
       <c r="A5" s="4" t="inlineStr">
         <is>
-          <t>גזרות</t>
+          <t>הגדוד הקולט</t>
         </is>
       </c>
       <c r="B5" s="11" t="n"/>
@@ -9369,7 +9369,7 @@
     <row r="6">
       <c r="A6" s="4" t="inlineStr">
         <is>
-          <t>גדוד מוסר א׳</t>
+          <t>מפקד הגדוד הקולט</t>
         </is>
       </c>
       <c r="B6" s="11" t="n"/>
@@ -9378,7 +9378,7 @@
     <row r="7">
       <c r="A7" s="4" t="inlineStr">
         <is>
-          <t>גדוד מוסר ב׳</t>
+          <t>גזרת גדס"ר</t>
         </is>
       </c>
       <c r="B7" s="11" t="n"/>
@@ -9387,7 +9387,7 @@
     <row r="8">
       <c r="A8" s="4" t="inlineStr">
         <is>
-          <t>הגדוד הקולט</t>
+          <t>גזרת 699</t>
         </is>
       </c>
       <c r="B8" s="11" t="n"/>
@@ -9396,181 +9396,195 @@
     <row r="9">
       <c r="A9" s="4" t="inlineStr">
         <is>
-          <t>מפקד הגדוד הקולט</t>
+          <t>תאריך ההעברה</t>
         </is>
       </c>
       <c r="B9" s="11" t="n"/>
       <c r="C9" s="12" t="n"/>
     </row>
-    <row r="10">
-      <c r="A10" s="4" t="inlineStr">
-        <is>
-          <t>תאריך ההעברה</t>
-        </is>
-      </c>
-      <c r="B10" s="11" t="n"/>
-      <c r="C10" s="12" t="n"/>
+    <row r="11">
+      <c r="A11" s="2" t="inlineStr">
+        <is>
+          <t>סיכום לפי גדוד מוסר (אוטומטי)</t>
+        </is>
+      </c>
     </row>
     <row r="12">
-      <c r="A12" s="2" t="inlineStr">
-        <is>
-          <t>סיכום לפי גדוד מוסר (אוטומטי)</t>
+      <c r="A12" s="3" t="inlineStr">
+        <is>
+          <t>גדוד מוסר</t>
+        </is>
+      </c>
+      <c r="B12" s="3" t="inlineStr">
+        <is>
+          <t>פריטים</t>
+        </is>
+      </c>
+      <c r="C12" s="3" t="inlineStr">
+        <is>
+          <t>כמות</t>
+        </is>
+      </c>
+      <c r="D12" s="3" t="inlineStr">
+        <is>
+          <t>פריטי צ׳</t>
+        </is>
+      </c>
+      <c r="E12" s="3" t="inlineStr">
+        <is>
+          <t>פערים</t>
         </is>
       </c>
     </row>
     <row r="13">
-      <c r="A13" s="3" t="inlineStr">
-        <is>
-          <t>גדוד מוסר</t>
-        </is>
-      </c>
-      <c r="B13" s="3" t="inlineStr">
-        <is>
-          <t>פריטים</t>
-        </is>
-      </c>
-      <c r="C13" s="3" t="inlineStr">
-        <is>
-          <t>כמות</t>
-        </is>
-      </c>
-      <c r="D13" s="3" t="inlineStr">
-        <is>
-          <t>פריטי צ׳</t>
-        </is>
-      </c>
-      <c r="E13" s="3" t="inlineStr">
-        <is>
-          <t>פערים</t>
-        </is>
+      <c r="A13" s="6">
+        <f>IF('מקרא והוראות'!$C$20="","",'מקרא והוראות'!$C$20)</f>
+        <v/>
+      </c>
+      <c r="B13" s="7">
+        <f>IF('מקרא והוראות'!$C$20="","",COUNTIF('רשימת ציוד'!$C$3:$C$302,'מקרא והוראות'!$C$20))</f>
+        <v/>
+      </c>
+      <c r="C13" s="7">
+        <f>IF('מקרא והוראות'!$C$20="","",SUMIF('רשימת ציוד'!$C$3:$C$302,'מקרא והוראות'!$C$20,'רשימת ציוד'!$I$3:$I$302))</f>
+        <v/>
+      </c>
+      <c r="D13" s="7">
+        <f>IF('מקרא והוראות'!$C$20="","",COUNTIFS('רשימת ציוד'!$C$3:$C$302,'מקרא והוראות'!$C$20,'רשימת ציוד'!$F$3:$F$302,"כן"))</f>
+        <v/>
+      </c>
+      <c r="E13" s="7">
+        <f>IF('מקרא והוראות'!$C$20="","",SUMPRODUCT(('רשימת ציוד'!$C$3:$C$302='מקרא והוראות'!$C$20)*('רשימת ציוד'!$L$3:$L$302&lt;&gt;"")*('רשימת ציוד'!$L$3:$L$302&lt;&gt;0)))</f>
+        <v/>
       </c>
     </row>
     <row r="14">
       <c r="A14" s="6">
-        <f>IF('מקרא והוראות'!$C$20="","",'מקרא והוראות'!$C$20)</f>
+        <f>IF('מקרא והוראות'!$C$21="","",'מקרא והוראות'!$C$21)</f>
         <v/>
       </c>
       <c r="B14" s="7">
-        <f>IF('מקרא והוראות'!$C$20="","",COUNTIF('רשימת ציוד'!$C$3:$C$302,'מקרא והוראות'!$C$20))</f>
+        <f>IF('מקרא והוראות'!$C$21="","",COUNTIF('רשימת ציוד'!$C$3:$C$302,'מקרא והוראות'!$C$21))</f>
         <v/>
       </c>
       <c r="C14" s="7">
-        <f>IF('מקרא והוראות'!$C$20="","",SUMIF('רשימת ציוד'!$C$3:$C$302,'מקרא והוראות'!$C$20,'רשימת ציוד'!$I$3:$I$302))</f>
+        <f>IF('מקרא והוראות'!$C$21="","",SUMIF('רשימת ציוד'!$C$3:$C$302,'מקרא והוראות'!$C$21,'רשימת ציוד'!$I$3:$I$302))</f>
         <v/>
       </c>
       <c r="D14" s="7">
-        <f>IF('מקרא והוראות'!$C$20="","",COUNTIFS('רשימת ציוד'!$C$3:$C$302,'מקרא והוראות'!$C$20,'רשימת ציוד'!$F$3:$F$302,"כן"))</f>
+        <f>IF('מקרא והוראות'!$C$21="","",COUNTIFS('רשימת ציוד'!$C$3:$C$302,'מקרא והוראות'!$C$21,'רשימת ציוד'!$F$3:$F$302,"כן"))</f>
         <v/>
       </c>
       <c r="E14" s="7">
-        <f>IF('מקרא והוראות'!$C$20="","",SUMPRODUCT(('רשימת ציוד'!$C$3:$C$302='מקרא והוראות'!$C$20)*('רשימת ציוד'!$L$3:$L$302&lt;&gt;"")*('רשימת ציוד'!$L$3:$L$302&lt;&gt;0)))</f>
+        <f>IF('מקרא והוראות'!$C$21="","",SUMPRODUCT(('רשימת ציוד'!$C$3:$C$302='מקרא והוראות'!$C$21)*('רשימת ציוד'!$L$3:$L$302&lt;&gt;"")*('רשימת ציוד'!$L$3:$L$302&lt;&gt;0)))</f>
         <v/>
       </c>
     </row>
     <row r="15">
       <c r="A15" s="6">
-        <f>IF('מקרא והוראות'!$C$21="","",'מקרא והוראות'!$C$21)</f>
+        <f>IF('מקרא והוראות'!$C$22="","",'מקרא והוראות'!$C$22)</f>
         <v/>
       </c>
       <c r="B15" s="7">
-        <f>IF('מקרא והוראות'!$C$21="","",COUNTIF('רשימת ציוד'!$C$3:$C$302,'מקרא והוראות'!$C$21))</f>
+        <f>IF('מקרא והוראות'!$C$22="","",COUNTIF('רשימת ציוד'!$C$3:$C$302,'מקרא והוראות'!$C$22))</f>
         <v/>
       </c>
       <c r="C15" s="7">
-        <f>IF('מקרא והוראות'!$C$21="","",SUMIF('רשימת ציוד'!$C$3:$C$302,'מקרא והוראות'!$C$21,'רשימת ציוד'!$I$3:$I$302))</f>
+        <f>IF('מקרא והוראות'!$C$22="","",SUMIF('רשימת ציוד'!$C$3:$C$302,'מקרא והוראות'!$C$22,'רשימת ציוד'!$I$3:$I$302))</f>
         <v/>
       </c>
       <c r="D15" s="7">
-        <f>IF('מקרא והוראות'!$C$21="","",COUNTIFS('רשימת ציוד'!$C$3:$C$302,'מקרא והוראות'!$C$21,'רשימת ציוד'!$F$3:$F$302,"כן"))</f>
+        <f>IF('מקרא והוראות'!$C$22="","",COUNTIFS('רשימת ציוד'!$C$3:$C$302,'מקרא והוראות'!$C$22,'רשימת ציוד'!$F$3:$F$302,"כן"))</f>
         <v/>
       </c>
       <c r="E15" s="7">
-        <f>IF('מקרא והוראות'!$C$21="","",SUMPRODUCT(('רשימת ציוד'!$C$3:$C$302='מקרא והוראות'!$C$21)*('רשימת ציוד'!$L$3:$L$302&lt;&gt;"")*('רשימת ציוד'!$L$3:$L$302&lt;&gt;0)))</f>
+        <f>IF('מקרא והוראות'!$C$22="","",SUMPRODUCT(('רשימת ציוד'!$C$3:$C$302='מקרא והוראות'!$C$22)*('רשימת ציוד'!$L$3:$L$302&lt;&gt;"")*('רשימת ציוד'!$L$3:$L$302&lt;&gt;0)))</f>
         <v/>
       </c>
     </row>
     <row r="16">
       <c r="A16" s="6">
-        <f>IF('מקרא והוראות'!$C$22="","",'מקרא והוראות'!$C$22)</f>
+        <f>IF('מקרא והוראות'!$C$23="","",'מקרא והוראות'!$C$23)</f>
         <v/>
       </c>
       <c r="B16" s="7">
-        <f>IF('מקרא והוראות'!$C$22="","",COUNTIF('רשימת ציוד'!$C$3:$C$302,'מקרא והוראות'!$C$22))</f>
+        <f>IF('מקרא והוראות'!$C$23="","",COUNTIF('רשימת ציוד'!$C$3:$C$302,'מקרא והוראות'!$C$23))</f>
         <v/>
       </c>
       <c r="C16" s="7">
-        <f>IF('מקרא והוראות'!$C$22="","",SUMIF('רשימת ציוד'!$C$3:$C$302,'מקרא והוראות'!$C$22,'רשימת ציוד'!$I$3:$I$302))</f>
+        <f>IF('מקרא והוראות'!$C$23="","",SUMIF('רשימת ציוד'!$C$3:$C$302,'מקרא והוראות'!$C$23,'רשימת ציוד'!$I$3:$I$302))</f>
         <v/>
       </c>
       <c r="D16" s="7">
-        <f>IF('מקרא והוראות'!$C$22="","",COUNTIFS('רשימת ציוד'!$C$3:$C$302,'מקרא והוראות'!$C$22,'רשימת ציוד'!$F$3:$F$302,"כן"))</f>
+        <f>IF('מקרא והוראות'!$C$23="","",COUNTIFS('רשימת ציוד'!$C$3:$C$302,'מקרא והוראות'!$C$23,'רשימת ציוד'!$F$3:$F$302,"כן"))</f>
         <v/>
       </c>
       <c r="E16" s="7">
-        <f>IF('מקרא והוראות'!$C$22="","",SUMPRODUCT(('רשימת ציוד'!$C$3:$C$302='מקרא והוראות'!$C$22)*('רשימת ציוד'!$L$3:$L$302&lt;&gt;"")*('רשימת ציוד'!$L$3:$L$302&lt;&gt;0)))</f>
-        <v/>
-      </c>
-    </row>
-    <row r="17">
-      <c r="A17" s="6">
-        <f>IF('מקרא והוראות'!$C$23="","",'מקרא והוראות'!$C$23)</f>
-        <v/>
-      </c>
-      <c r="B17" s="7">
-        <f>IF('מקרא והוראות'!$C$23="","",COUNTIF('רשימת ציוד'!$C$3:$C$302,'מקרא והוראות'!$C$23))</f>
-        <v/>
-      </c>
-      <c r="C17" s="7">
-        <f>IF('מקרא והוראות'!$C$23="","",SUMIF('רשימת ציוד'!$C$3:$C$302,'מקרא והוראות'!$C$23,'רשימת ציוד'!$I$3:$I$302))</f>
-        <v/>
-      </c>
-      <c r="D17" s="7">
-        <f>IF('מקרא והוראות'!$C$23="","",COUNTIFS('רשימת ציוד'!$C$3:$C$302,'מקרא והוראות'!$C$23,'רשימת ציוד'!$F$3:$F$302,"כן"))</f>
-        <v/>
-      </c>
-      <c r="E17" s="7">
         <f>IF('מקרא והוראות'!$C$23="","",SUMPRODUCT(('רשימת ציוד'!$C$3:$C$302='מקרא והוראות'!$C$23)*('רשימת ציוד'!$L$3:$L$302&lt;&gt;"")*('רשימת ציוד'!$L$3:$L$302&lt;&gt;0)))</f>
         <v/>
       </c>
     </row>
+    <row r="18">
+      <c r="A18" s="2" t="inlineStr">
+        <is>
+          <t>סיכום לפי קטגוריה (אוטומטי)</t>
+        </is>
+      </c>
+    </row>
     <row r="19">
-      <c r="A19" s="2" t="inlineStr">
-        <is>
-          <t>סיכום לפי קטגוריה (אוטומטי)</t>
+      <c r="A19" s="3" t="inlineStr">
+        <is>
+          <t>קטגוריה</t>
+        </is>
+      </c>
+      <c r="B19" s="3" t="inlineStr">
+        <is>
+          <t>פריטים</t>
+        </is>
+      </c>
+      <c r="C19" s="3" t="inlineStr">
+        <is>
+          <t>כמות</t>
+        </is>
+      </c>
+      <c r="D19" s="3" t="inlineStr">
+        <is>
+          <t>פריטי צ׳</t>
+        </is>
+      </c>
+      <c r="E19" s="3" t="inlineStr">
+        <is>
+          <t>פערים</t>
         </is>
       </c>
     </row>
     <row r="20">
-      <c r="A20" s="3" t="inlineStr">
-        <is>
-          <t>קטגוריה</t>
-        </is>
-      </c>
-      <c r="B20" s="3" t="inlineStr">
-        <is>
-          <t>פריטים</t>
-        </is>
-      </c>
-      <c r="C20" s="3" t="inlineStr">
-        <is>
-          <t>כמות</t>
-        </is>
-      </c>
-      <c r="D20" s="3" t="inlineStr">
-        <is>
-          <t>פריטי צ׳</t>
-        </is>
-      </c>
-      <c r="E20" s="3" t="inlineStr">
-        <is>
-          <t>פערים</t>
-        </is>
+      <c r="A20" s="6" t="inlineStr">
+        <is>
+          <t>אמל"ח</t>
+        </is>
+      </c>
+      <c r="B20" s="7">
+        <f>COUNTIF('רשימת ציוד'!$D$3:$D$302,$A20)</f>
+        <v/>
+      </c>
+      <c r="C20" s="7">
+        <f>SUMIF('רשימת ציוד'!$D$3:$D$302,$A20,'רשימת ציוד'!$I$3:$I$302)</f>
+        <v/>
+      </c>
+      <c r="D20" s="7">
+        <f>COUNTIFS('רשימת ציוד'!$D$3:$D$302,$A20,'רשימת ציוד'!$F$3:$F$302,"כן")</f>
+        <v/>
+      </c>
+      <c r="E20" s="7">
+        <f>SUMPRODUCT(('רשימת ציוד'!$D$3:$D$302=$A20)*('רשימת ציוד'!$L$3:$L$302&lt;&gt;"")*('רשימת ציוד'!$L$3:$L$302&lt;&gt;0))</f>
+        <v/>
       </c>
     </row>
     <row r="21">
       <c r="A21" s="6" t="inlineStr">
         <is>
-          <t>אמל"ח</t>
+          <t>תחמושת</t>
         </is>
       </c>
       <c r="B21" s="7">
@@ -9593,7 +9607,7 @@
     <row r="22">
       <c r="A22" s="6" t="inlineStr">
         <is>
-          <t>תחמושת</t>
+          <t>אופטיקה ותצפית</t>
         </is>
       </c>
       <c r="B22" s="7">
@@ -9616,7 +9630,7 @@
     <row r="23">
       <c r="A23" s="6" t="inlineStr">
         <is>
-          <t>אופטיקה ותצפית</t>
+          <t>קשר ומחשוב</t>
         </is>
       </c>
       <c r="B23" s="7">
@@ -9639,7 +9653,7 @@
     <row r="24">
       <c r="A24" s="6" t="inlineStr">
         <is>
-          <t>קשר ומחשוב</t>
+          <t>רחפנים</t>
         </is>
       </c>
       <c r="B24" s="7">
@@ -9662,7 +9676,7 @@
     <row r="25">
       <c r="A25" s="6" t="inlineStr">
         <is>
-          <t>רחפנים</t>
+          <t>מיגון</t>
         </is>
       </c>
       <c r="B25" s="7">
@@ -9685,7 +9699,7 @@
     <row r="26">
       <c r="A26" s="6" t="inlineStr">
         <is>
-          <t>מיגון</t>
+          <t>ציוד רפואי</t>
         </is>
       </c>
       <c r="B26" s="7">
@@ -9708,7 +9722,7 @@
     <row r="27">
       <c r="A27" s="6" t="inlineStr">
         <is>
-          <t>ציוד רפואי</t>
+          <t>לוגיסטיקה ומגורים</t>
         </is>
       </c>
       <c r="B27" s="7">
@@ -9731,7 +9745,7 @@
     <row r="28">
       <c r="A28" s="6" t="inlineStr">
         <is>
-          <t>לוגיסטיקה ומגורים</t>
+          <t>מטבח ומזון</t>
         </is>
       </c>
       <c r="B28" s="7">
@@ -9754,7 +9768,7 @@
     <row r="29">
       <c r="A29" s="6" t="inlineStr">
         <is>
-          <t>מטבח ומזון</t>
+          <t>גנרטורים וחשמל</t>
         </is>
       </c>
       <c r="B29" s="7">
@@ -9777,7 +9791,7 @@
     <row r="30">
       <c r="A30" s="6" t="inlineStr">
         <is>
-          <t>גנרטורים וחשמל</t>
+          <t>תשתיות ומבנה</t>
         </is>
       </c>
       <c r="B30" s="7">
@@ -9800,7 +9814,7 @@
     <row r="31">
       <c r="A31" s="6" t="inlineStr">
         <is>
-          <t>תשתיות ומבנה</t>
+          <t>כיבוי אש ובטיחות</t>
         </is>
       </c>
       <c r="B31" s="7">
@@ -9823,7 +9837,7 @@
     <row r="32">
       <c r="A32" s="6" t="inlineStr">
         <is>
-          <t>כיבוי אש ובטיחות</t>
+          <t>אחר</t>
         </is>
       </c>
       <c r="B32" s="7">
@@ -9844,136 +9858,125 @@
       </c>
     </row>
     <row r="33">
-      <c r="A33" s="6" t="inlineStr">
-        <is>
-          <t>אחר</t>
-        </is>
-      </c>
-      <c r="B33" s="7">
-        <f>COUNTIF('רשימת ציוד'!$D$3:$D$302,$A33)</f>
-        <v/>
-      </c>
-      <c r="C33" s="7">
-        <f>SUMIF('רשימת ציוד'!$D$3:$D$302,$A33,'רשימת ציוד'!$I$3:$I$302)</f>
-        <v/>
-      </c>
-      <c r="D33" s="7">
-        <f>COUNTIFS('רשימת ציוד'!$D$3:$D$302,$A33,'רשימת ציוד'!$F$3:$F$302,"כן")</f>
-        <v/>
-      </c>
-      <c r="E33" s="7">
-        <f>SUMPRODUCT(('רשימת ציוד'!$D$3:$D$302=$A33)*('רשימת ציוד'!$L$3:$L$302&lt;&gt;"")*('רשימת ציוד'!$L$3:$L$302&lt;&gt;0))</f>
-        <v/>
-      </c>
-    </row>
-    <row r="34">
-      <c r="A34" s="10" t="inlineStr">
+      <c r="A33" s="10" t="inlineStr">
         <is>
           <t>סה"כ</t>
         </is>
       </c>
-      <c r="B34" s="10">
-        <f>SUM(B21:B33)</f>
-        <v/>
-      </c>
-      <c r="C34" s="10">
-        <f>SUM(C21:C33)</f>
-        <v/>
-      </c>
-      <c r="D34" s="10">
-        <f>SUM(D21:D33)</f>
-        <v/>
-      </c>
-      <c r="E34" s="10">
-        <f>SUM(E21:E33)</f>
-        <v/>
+      <c r="B33" s="10">
+        <f>SUM(B20:B32)</f>
+        <v/>
+      </c>
+      <c r="C33" s="10">
+        <f>SUM(C20:C32)</f>
+        <v/>
+      </c>
+      <c r="D33" s="10">
+        <f>SUM(D20:D32)</f>
+        <v/>
+      </c>
+      <c r="E33" s="10">
+        <f>SUM(E20:E32)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="35">
+      <c r="A35" s="2" t="inlineStr">
+        <is>
+          <t>הצהרה</t>
+        </is>
       </c>
     </row>
     <row r="36">
-      <c r="A36" s="2" t="inlineStr">
-        <is>
-          <t>הצהרה</t>
+      <c r="A36" s="13" t="inlineStr">
+        <is>
+          <t>אנו החתומים מטה מאשרים כי:</t>
         </is>
       </c>
     </row>
     <row r="37">
       <c r="A37" s="13" t="inlineStr">
         <is>
-          <t>אנו החתומים מטה מאשרים כי:</t>
+          <t>1. הציוד המפורט בגיליון 'רשימת ציוד' נספר ונבדק במעמד נציגי הגדודים המוסרים והגדוד הקולט.</t>
         </is>
       </c>
     </row>
     <row r="38">
       <c r="A38" s="13" t="inlineStr">
         <is>
-          <t>1. הציוד המפורט בגיליון 'רשימת ציוד' נספר ונבדק במעמד נציגי הגדודים המוסרים והגדוד הקולט.</t>
+          <t>2. הגדוד הקולט מאשר את קבלת הציוד בכמויות ובמצב כמפורט, למעט הפערים שצוינו.</t>
         </is>
       </c>
     </row>
     <row r="39">
       <c r="A39" s="13" t="inlineStr">
         <is>
-          <t>2. הגדוד הקולט מאשר את קבלת הציוד בכמויות ובמצב כמפורט, למעט הפערים שצוינו.</t>
+          <t>3. פערים שנרשמו יתועדו ויטופלו מול החטיבה.</t>
         </is>
       </c>
     </row>
     <row r="40">
       <c r="A40" s="13" t="inlineStr">
         <is>
-          <t>3. פערים שנרשמו יתועדו ויטופלו מול החטיבה.</t>
-        </is>
-      </c>
-    </row>
-    <row r="41">
-      <c r="A41" s="13" t="inlineStr">
-        <is>
           <t>4. האחריות על הציוד, לרבות פריטי הצ׳, עוברת לגדוד הקולט מרגע החתימה.</t>
         </is>
       </c>
     </row>
+    <row r="42">
+      <c r="A42" s="2" t="inlineStr">
+        <is>
+          <t>חתימות</t>
+        </is>
+      </c>
+    </row>
     <row r="43">
-      <c r="A43" s="2" t="inlineStr">
-        <is>
-          <t>חתימות</t>
-        </is>
-      </c>
-    </row>
-    <row r="44">
-      <c r="A44" s="3" t="inlineStr">
+      <c r="A43" s="3" t="inlineStr">
         <is>
           <t>תפקיד</t>
         </is>
       </c>
-      <c r="B44" s="3" t="inlineStr">
+      <c r="B43" s="3" t="inlineStr">
         <is>
           <t>שם מלא</t>
         </is>
       </c>
-      <c r="C44" s="3" t="inlineStr">
+      <c r="C43" s="3" t="inlineStr">
         <is>
           <t>דרגה</t>
         </is>
       </c>
-      <c r="D44" s="3" t="inlineStr">
+      <c r="D43" s="3" t="inlineStr">
         <is>
           <t>מס׳ אישי</t>
         </is>
       </c>
-      <c r="E44" s="3" t="inlineStr">
+      <c r="E43" s="3" t="inlineStr">
         <is>
           <t>תאריך</t>
         </is>
       </c>
-      <c r="F44" s="3" t="inlineStr">
+      <c r="F43" s="3" t="inlineStr">
         <is>
           <t>חתימה</t>
         </is>
       </c>
+    </row>
+    <row r="44" ht="24" customHeight="1">
+      <c r="A44" s="4" t="inlineStr">
+        <is>
+          <t>גדס"ר – מפקד</t>
+        </is>
+      </c>
+      <c r="B44" s="12" t="n"/>
+      <c r="C44" s="12" t="n"/>
+      <c r="D44" s="12" t="n"/>
+      <c r="E44" s="12" t="n"/>
+      <c r="F44" s="12" t="n"/>
     </row>
     <row r="45" ht="24" customHeight="1">
       <c r="A45" s="4" t="inlineStr">
         <is>
-          <t>גדוד מוסר א׳ – מפקד</t>
+          <t>גדס"ר – קצין לוגיסטיקה / אפסנאי</t>
         </is>
       </c>
       <c r="B45" s="12" t="n"/>
@@ -9985,7 +9988,7 @@
     <row r="46" ht="24" customHeight="1">
       <c r="A46" s="4" t="inlineStr">
         <is>
-          <t>גדוד מוסר א׳ – קצין לוגיסטיקה / אפסנאי</t>
+          <t>699 – מפקד</t>
         </is>
       </c>
       <c r="B46" s="12" t="n"/>
@@ -9997,7 +10000,7 @@
     <row r="47" ht="24" customHeight="1">
       <c r="A47" s="4" t="inlineStr">
         <is>
-          <t>גדוד מוסר ב׳ – מפקד</t>
+          <t>699 – קצין לוגיסטיקה / אפסנאי</t>
         </is>
       </c>
       <c r="B47" s="12" t="n"/>
@@ -10009,7 +10012,7 @@
     <row r="48" ht="24" customHeight="1">
       <c r="A48" s="4" t="inlineStr">
         <is>
-          <t>גדוד מוסר ב׳ – קצין לוגיסטיקה / אפסנאי</t>
+          <t>הגדוד הקולט – מפקד</t>
         </is>
       </c>
       <c r="B48" s="12" t="n"/>
@@ -10021,7 +10024,7 @@
     <row r="49" ht="24" customHeight="1">
       <c r="A49" s="4" t="inlineStr">
         <is>
-          <t>הגדוד הקולט – מפקד</t>
+          <t>הגדוד הקולט – קצין לוגיסטיקה / אפסנאי</t>
         </is>
       </c>
       <c r="B49" s="12" t="n"/>
@@ -10033,7 +10036,7 @@
     <row r="50" ht="24" customHeight="1">
       <c r="A50" s="4" t="inlineStr">
         <is>
-          <t>הגדוד הקולט – קצין לוגיסטיקה / אפסנאי</t>
+          <t>נציג חטיבה</t>
         </is>
       </c>
       <c r="B50" s="12" t="n"/>
@@ -10042,41 +10045,28 @@
       <c r="E50" s="12" t="n"/>
       <c r="F50" s="12" t="n"/>
     </row>
-    <row r="51" ht="24" customHeight="1">
-      <c r="A51" s="4" t="inlineStr">
-        <is>
-          <t>נציג חטיבה</t>
-        </is>
-      </c>
-      <c r="B51" s="12" t="n"/>
-      <c r="C51" s="12" t="n"/>
-      <c r="D51" s="12" t="n"/>
-      <c r="E51" s="12" t="n"/>
-      <c r="F51" s="12" t="n"/>
-    </row>
-    <row r="53">
-      <c r="A53" s="13" t="inlineStr">
+    <row r="52">
+      <c r="A52" s="13" t="inlineStr">
         <is>
           <t>* מומלץ להדפיס עותק לכל גדוד מוסר + עותק לגדוד הקולט.</t>
         </is>
       </c>
     </row>
   </sheetData>
-  <mergeCells count="14">
+  <mergeCells count="13">
     <mergeCell ref="A38:F38"/>
-    <mergeCell ref="A41:F41"/>
     <mergeCell ref="B6:C6"/>
+    <mergeCell ref="A52:F52"/>
     <mergeCell ref="B7:C7"/>
+    <mergeCell ref="A36:F36"/>
     <mergeCell ref="B5:C5"/>
     <mergeCell ref="A1:F1"/>
     <mergeCell ref="A37:F37"/>
-    <mergeCell ref="B10:C10"/>
     <mergeCell ref="A40:F40"/>
     <mergeCell ref="B9:C9"/>
     <mergeCell ref="B8:C8"/>
     <mergeCell ref="B4:C4"/>
     <mergeCell ref="A39:F39"/>
-    <mergeCell ref="A53:F53"/>
   </mergeCells>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
   <pageSetup fitToHeight="1" fitToWidth="1"/>
@@ -10220,7 +10210,7 @@
       </c>
       <c r="C20" s="7" t="inlineStr">
         <is>
-          <t>גדוד א׳</t>
+          <t>גדס"ר</t>
         </is>
       </c>
     </row>
@@ -10232,7 +10222,7 @@
       </c>
       <c r="C21" s="7" t="inlineStr">
         <is>
-          <t>גדוד ב׳</t>
+          <t>699</t>
         </is>
       </c>
     </row>

</xml_diff>